<commit_message>
new data changed some directories
</commit_message>
<xml_diff>
--- a/data/belt_mine.xlsx
+++ b/data/belt_mine.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="10" documentId="11_1D1A589243950EE2E86E6420DA7D1FB1B490D5A9" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0C055712-FE7E-7D4A-81AD-9D4712FE2E14}"/>
   <bookViews>
-    <workbookView xWindow="33720" yWindow="3860" windowWidth="29400" windowHeight="16720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="33720" yWindow="3900" windowWidth="29400" windowHeight="16720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BC" sheetId="1" r:id="rId1"/>
@@ -321,6 +321,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>